<commit_message>
Auto backup 2026-07-02 07:05:02
</commit_message>
<xml_diff>
--- a/SwissTechShehzad/1-07-2026/jbl.xlsx
+++ b/SwissTechShehzad/1-07-2026/jbl.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\1-07-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C7BF0294-E817-4141-9E20-F7144A003542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CCBA1D1-79AA-485A-8A9C-F3137B506258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28692" yWindow="-1896" windowWidth="29016" windowHeight="17496" xr2:uid="{DD915E75-360C-4CDB-9DCF-0FF792C624AE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DD915E75-360C-4CDB-9DCF-0FF792C624AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t xml:space="preserve">S NO </t>
   </si>
@@ -57,13 +57,7 @@
     <t>webite in australia</t>
   </si>
   <si>
-    <t>harveynorman.com.au</t>
-  </si>
-  <si>
     <t>price</t>
-  </si>
-  <si>
-    <t>jbhifi.com.au</t>
   </si>
 </sst>
 </file>
@@ -122,10 +116,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -458,7 +452,7 @@
         <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -485,28 +479,20 @@
       <c r="C4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="4">
-        <v>283</v>
-      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="4">
-        <v>299</v>
-      </c>
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>